<commit_message>
finish change setup and add galadinner setting
</commit_message>
<xml_diff>
--- a/test files/New year galadinner.xlsx
+++ b/test files/New year galadinner.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\batcave\work\Credit_App\Credit_app_v3_test\test files\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E54C0587-B7DE-4948-B064-66B7275799C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="75" windowWidth="15480" windowHeight="10920"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="statment" sheetId="6" r:id="rId1"/>
@@ -20,14 +26,27 @@
     <externalReference r:id="rId9"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">statment!$B$1:$J$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">statment!$B$1:$K$19</definedName>
   </definedNames>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="22">
   <si>
     <t>Night</t>
   </si>
@@ -91,11 +110,14 @@
   <si>
     <t>102-126</t>
   </si>
+  <si>
+    <t>pax</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;_-* #,##0.00\-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy;@"/>
@@ -458,7 +480,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -567,55 +589,66 @@
     <xf numFmtId="164" fontId="13" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="1" fontId="5" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="44">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 10 2" xfId="2"/>
-    <cellStyle name="Normal 10 3" xfId="3"/>
-    <cellStyle name="Normal 10 4" xfId="4"/>
-    <cellStyle name="Normal 140" xfId="5"/>
-    <cellStyle name="Normal 148" xfId="6"/>
-    <cellStyle name="Normal 149" xfId="7"/>
-    <cellStyle name="Normal 151" xfId="8"/>
-    <cellStyle name="Normal 152" xfId="40"/>
-    <cellStyle name="Normal 153" xfId="9"/>
-    <cellStyle name="Normal 154" xfId="10"/>
-    <cellStyle name="Normal 157" xfId="38"/>
-    <cellStyle name="Normal 158" xfId="39"/>
-    <cellStyle name="Normal 159" xfId="11"/>
-    <cellStyle name="Normal 160" xfId="12"/>
-    <cellStyle name="Normal 162" xfId="13"/>
-    <cellStyle name="Normal 163" xfId="14"/>
-    <cellStyle name="Normal 165" xfId="15"/>
-    <cellStyle name="Normal 166" xfId="16"/>
-    <cellStyle name="Normal 19 2" xfId="17"/>
-    <cellStyle name="Normal 19 3" xfId="18"/>
-    <cellStyle name="Normal 19 4" xfId="19"/>
-    <cellStyle name="Normal 2" xfId="43"/>
-    <cellStyle name="Normal 2 2" xfId="20"/>
-    <cellStyle name="Normal 2 3" xfId="21"/>
-    <cellStyle name="Normal 2 4" xfId="22"/>
-    <cellStyle name="Normal 20 2" xfId="23"/>
-    <cellStyle name="Normal 20 3" xfId="24"/>
-    <cellStyle name="Normal 20 4" xfId="25"/>
-    <cellStyle name="Normal 23 2" xfId="26"/>
-    <cellStyle name="Normal 23 3" xfId="27"/>
-    <cellStyle name="Normal 23 4" xfId="28"/>
-    <cellStyle name="Normal 3" xfId="41"/>
-    <cellStyle name="Normal 37 2" xfId="29"/>
-    <cellStyle name="Normal 37 3" xfId="30"/>
-    <cellStyle name="Normal 37 4" xfId="31"/>
-    <cellStyle name="Normal 38 2" xfId="32"/>
-    <cellStyle name="Normal 38 3" xfId="33"/>
-    <cellStyle name="Normal 38 4" xfId="34"/>
-    <cellStyle name="Normal 5" xfId="42"/>
-    <cellStyle name="Normal 9 2" xfId="35"/>
-    <cellStyle name="Normal 9 3" xfId="36"/>
-    <cellStyle name="Normal 9 4" xfId="37"/>
+    <cellStyle name="Normal 10 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
+    <cellStyle name="Normal 10 3" xfId="3" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
+    <cellStyle name="Normal 10 4" xfId="4" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
+    <cellStyle name="Normal 140" xfId="5" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
+    <cellStyle name="Normal 148" xfId="6" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
+    <cellStyle name="Normal 149" xfId="7" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
+    <cellStyle name="Normal 151" xfId="8" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
+    <cellStyle name="Normal 152" xfId="40" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
+    <cellStyle name="Normal 153" xfId="9" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
+    <cellStyle name="Normal 154" xfId="10" xr:uid="{00000000-0005-0000-0000-00000B000000}"/>
+    <cellStyle name="Normal 157" xfId="38" xr:uid="{00000000-0005-0000-0000-00000C000000}"/>
+    <cellStyle name="Normal 158" xfId="39" xr:uid="{00000000-0005-0000-0000-00000D000000}"/>
+    <cellStyle name="Normal 159" xfId="11" xr:uid="{00000000-0005-0000-0000-00000E000000}"/>
+    <cellStyle name="Normal 160" xfId="12" xr:uid="{00000000-0005-0000-0000-00000F000000}"/>
+    <cellStyle name="Normal 162" xfId="13" xr:uid="{00000000-0005-0000-0000-000010000000}"/>
+    <cellStyle name="Normal 163" xfId="14" xr:uid="{00000000-0005-0000-0000-000011000000}"/>
+    <cellStyle name="Normal 165" xfId="15" xr:uid="{00000000-0005-0000-0000-000012000000}"/>
+    <cellStyle name="Normal 166" xfId="16" xr:uid="{00000000-0005-0000-0000-000013000000}"/>
+    <cellStyle name="Normal 19 2" xfId="17" xr:uid="{00000000-0005-0000-0000-000014000000}"/>
+    <cellStyle name="Normal 19 3" xfId="18" xr:uid="{00000000-0005-0000-0000-000015000000}"/>
+    <cellStyle name="Normal 19 4" xfId="19" xr:uid="{00000000-0005-0000-0000-000016000000}"/>
+    <cellStyle name="Normal 2" xfId="43" xr:uid="{00000000-0005-0000-0000-000017000000}"/>
+    <cellStyle name="Normal 2 2" xfId="20" xr:uid="{00000000-0005-0000-0000-000018000000}"/>
+    <cellStyle name="Normal 2 3" xfId="21" xr:uid="{00000000-0005-0000-0000-000019000000}"/>
+    <cellStyle name="Normal 2 4" xfId="22" xr:uid="{00000000-0005-0000-0000-00001A000000}"/>
+    <cellStyle name="Normal 20 2" xfId="23" xr:uid="{00000000-0005-0000-0000-00001B000000}"/>
+    <cellStyle name="Normal 20 3" xfId="24" xr:uid="{00000000-0005-0000-0000-00001C000000}"/>
+    <cellStyle name="Normal 20 4" xfId="25" xr:uid="{00000000-0005-0000-0000-00001D000000}"/>
+    <cellStyle name="Normal 23 2" xfId="26" xr:uid="{00000000-0005-0000-0000-00001E000000}"/>
+    <cellStyle name="Normal 23 3" xfId="27" xr:uid="{00000000-0005-0000-0000-00001F000000}"/>
+    <cellStyle name="Normal 23 4" xfId="28" xr:uid="{00000000-0005-0000-0000-000020000000}"/>
+    <cellStyle name="Normal 3" xfId="41" xr:uid="{00000000-0005-0000-0000-000021000000}"/>
+    <cellStyle name="Normal 37 2" xfId="29" xr:uid="{00000000-0005-0000-0000-000022000000}"/>
+    <cellStyle name="Normal 37 3" xfId="30" xr:uid="{00000000-0005-0000-0000-000023000000}"/>
+    <cellStyle name="Normal 37 4" xfId="31" xr:uid="{00000000-0005-0000-0000-000024000000}"/>
+    <cellStyle name="Normal 38 2" xfId="32" xr:uid="{00000000-0005-0000-0000-000025000000}"/>
+    <cellStyle name="Normal 38 3" xfId="33" xr:uid="{00000000-0005-0000-0000-000026000000}"/>
+    <cellStyle name="Normal 38 4" xfId="34" xr:uid="{00000000-0005-0000-0000-000027000000}"/>
+    <cellStyle name="Normal 5" xfId="42" xr:uid="{00000000-0005-0000-0000-000028000000}"/>
+    <cellStyle name="Normal 9 2" xfId="35" xr:uid="{00000000-0005-0000-0000-000029000000}"/>
+    <cellStyle name="Normal 9 3" xfId="36" xr:uid="{00000000-0005-0000-0000-00002A000000}"/>
+    <cellStyle name="Normal 9 4" xfId="37" xr:uid="{00000000-0005-0000-0000-00002B000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -636,7 +669,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2049" name="Picture 1"/>
+        <xdr:cNvPr id="2049" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000001080000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
         </xdr:cNvPicPr>
@@ -676,7 +715,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2"/>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000003000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -719,7 +764,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Picture 4"/>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000005000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -757,7 +808,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2"/>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000003000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -795,7 +852,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3"/>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000004000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -838,7 +901,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1"/>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -876,7 +945,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3"/>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000004000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -914,7 +989,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="7" name="Picture 6"/>
+        <xdr:cNvPr id="7" name="Picture 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000007000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -952,7 +1033,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="9" name="Picture 8"/>
+        <xdr:cNvPr id="9" name="Picture 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000009000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -990,7 +1077,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Picture 5"/>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000006000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -1033,7 +1126,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2"/>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0400-000003000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -1060,7 +1159,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Dec 24"/>
@@ -1079,7 +1178,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Feb 2024"/>
@@ -1100,7 +1199,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Dec 24"/>
@@ -1115,7 +1214,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink4.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Dec 24"/>
@@ -1132,9 +1231,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1172,7 +1271,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -1206,6 +1305,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -1240,9 +1340,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1415,20 +1516,21 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J19"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:K19"/>
+  <sheetFormatPr defaultRowHeight="13.2"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" customWidth="1"/>
-    <col min="2" max="2" width="24.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.7109375" customWidth="1"/>
-    <col min="4" max="4" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="20.7109375" customWidth="1"/>
+    <col min="1" max="1" width="20.6640625" customWidth="1"/>
+    <col min="2" max="2" width="24.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.6640625" customWidth="1"/>
+    <col min="4" max="4" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="20.6640625" customWidth="1"/>
     <col min="7" max="7" width="24" bestFit="1" customWidth="1"/>
-    <col min="8" max="10" width="20.7109375" customWidth="1"/>
+    <col min="8" max="8" width="24" customWidth="1"/>
+    <col min="9" max="11" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="20.25" thickTop="1" thickBot="1">
+    <row r="1" spans="1:11" ht="18.600000000000001" thickTop="1" thickBot="1">
       <c r="B1" s="3" t="s">
         <v>9</v>
       </c>
@@ -1447,17 +1549,20 @@
       <c r="G1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:10" s="21" customFormat="1" ht="16.5" thickTop="1">
+    <row r="2" spans="1:11" s="21" customFormat="1" ht="16.2" thickTop="1">
       <c r="A2" s="20"/>
       <c r="B2" s="28">
         <v>10918056</v>
@@ -1477,18 +1582,21 @@
       <c r="G2" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="H2" s="32">
-        <f t="shared" ref="H2:H19" si="0">+F2-E2</f>
+      <c r="H2" s="42">
+        <v>1</v>
+      </c>
+      <c r="I2" s="32">
+        <f t="shared" ref="I2:I19" si="0">+F2-E2</f>
         <v>10</v>
       </c>
-      <c r="I2" s="33">
+      <c r="J2" s="33">
         <v>58</v>
       </c>
-      <c r="J2" s="34">
+      <c r="K2" s="34">
         <v>580</v>
       </c>
     </row>
-    <row r="3" spans="1:10" s="21" customFormat="1" ht="15.75">
+    <row r="3" spans="1:11" s="21" customFormat="1" ht="15.6">
       <c r="A3" s="20"/>
       <c r="B3" s="35">
         <v>10929447</v>
@@ -1508,18 +1616,21 @@
       <c r="G3" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="H3" s="39">
+      <c r="H3" s="42">
+        <v>2</v>
+      </c>
+      <c r="I3" s="39">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="I3" s="40">
+      <c r="J3" s="40">
         <v>72</v>
       </c>
-      <c r="J3" s="41">
+      <c r="K3" s="41">
         <v>504</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="15.75">
+    <row r="4" spans="1:11" ht="15.6">
       <c r="B4" s="35">
         <v>10944993</v>
       </c>
@@ -1538,18 +1649,21 @@
       <c r="G4" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="H4" s="39">
+      <c r="H4" s="42">
+        <v>2</v>
+      </c>
+      <c r="I4" s="39">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="I4" s="40">
+      <c r="J4" s="40">
         <v>60</v>
       </c>
-      <c r="J4" s="41">
+      <c r="K4" s="41">
         <v>720</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="15.75">
+    <row r="5" spans="1:11" ht="15.6">
       <c r="B5" s="35">
         <v>10948811</v>
       </c>
@@ -1568,18 +1682,21 @@
       <c r="G5" s="38" t="s">
         <v>16</v>
       </c>
-      <c r="H5" s="39">
+      <c r="H5" s="42">
+        <v>3</v>
+      </c>
+      <c r="I5" s="39">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="I5" s="40">
+      <c r="J5" s="40">
         <v>81</v>
       </c>
-      <c r="J5" s="41">
+      <c r="K5" s="41">
         <v>810</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="15.75">
+    <row r="6" spans="1:11" ht="15.6">
       <c r="B6" s="35">
         <v>10947743</v>
       </c>
@@ -1598,18 +1715,21 @@
       <c r="G6" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="H6" s="39">
+      <c r="H6" s="42">
+        <v>1</v>
+      </c>
+      <c r="I6" s="39">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="I6" s="40">
+      <c r="J6" s="40">
         <v>60</v>
       </c>
-      <c r="J6" s="41">
+      <c r="K6" s="41">
         <v>660</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="15.75">
+    <row r="7" spans="1:11" ht="15.6">
       <c r="B7" s="35">
         <v>10947678</v>
       </c>
@@ -1628,18 +1748,21 @@
       <c r="G7" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="39">
+      <c r="H7" s="42">
+        <v>1</v>
+      </c>
+      <c r="I7" s="39">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="I7" s="40">
+      <c r="J7" s="40">
         <v>60</v>
       </c>
-      <c r="J7" s="41">
+      <c r="K7" s="41">
         <v>660</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="15.75">
+    <row r="8" spans="1:11" ht="15.6">
       <c r="B8" s="35">
         <v>10947681</v>
       </c>
@@ -1658,18 +1781,21 @@
       <c r="G8" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="H8" s="39">
+      <c r="H8" s="42">
+        <v>1</v>
+      </c>
+      <c r="I8" s="39">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="I8" s="40">
+      <c r="J8" s="40">
         <v>48</v>
       </c>
-      <c r="J8" s="41">
+      <c r="K8" s="41">
         <v>528</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="15.75">
+    <row r="9" spans="1:11" ht="15.6">
       <c r="B9" s="35">
         <v>10948453</v>
       </c>
@@ -1688,18 +1814,21 @@
       <c r="G9" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="H9" s="39">
+      <c r="H9" s="42">
+        <v>1</v>
+      </c>
+      <c r="I9" s="39">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="I9" s="40">
+      <c r="J9" s="40">
         <v>60</v>
       </c>
-      <c r="J9" s="41">
+      <c r="K9" s="41">
         <v>660</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="15.75">
+    <row r="10" spans="1:11" ht="15.6">
       <c r="B10" s="35">
         <v>10952417</v>
       </c>
@@ -1718,18 +1847,21 @@
       <c r="G10" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="H10" s="39">
+      <c r="H10" s="42">
+        <v>1</v>
+      </c>
+      <c r="I10" s="39">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="I10" s="40">
+      <c r="J10" s="40">
         <v>48</v>
       </c>
-      <c r="J10" s="41">
+      <c r="K10" s="41">
         <v>192</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="15.75">
+    <row r="11" spans="1:11" ht="15.6">
       <c r="B11" s="35">
         <v>10829403</v>
       </c>
@@ -1748,18 +1880,21 @@
       <c r="G11" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="H11" s="39">
+      <c r="H11" s="42">
+        <v>1</v>
+      </c>
+      <c r="I11" s="39">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="I11" s="40">
+      <c r="J11" s="40">
         <v>72</v>
       </c>
-      <c r="J11" s="41">
+      <c r="K11" s="41">
         <v>504</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="15.75">
+    <row r="12" spans="1:11" ht="15.6">
       <c r="B12" s="35">
         <v>10953390</v>
       </c>
@@ -1778,18 +1913,21 @@
       <c r="G12" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="H12" s="39">
+      <c r="H12" s="42">
+        <v>1</v>
+      </c>
+      <c r="I12" s="39">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="I12" s="40">
+      <c r="J12" s="40">
         <v>60</v>
       </c>
-      <c r="J12" s="41">
+      <c r="K12" s="41">
         <v>420</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="15.75">
+    <row r="13" spans="1:11" ht="15.6">
       <c r="B13" s="35">
         <v>10955653</v>
       </c>
@@ -1808,18 +1946,21 @@
       <c r="G13" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="H13" s="39">
+      <c r="H13" s="42">
+        <v>1</v>
+      </c>
+      <c r="I13" s="39">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="I13" s="40">
+      <c r="J13" s="40">
         <v>92.5</v>
       </c>
-      <c r="J13" s="41">
+      <c r="K13" s="41">
         <v>925</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="15.75">
+    <row r="14" spans="1:11" ht="15.6">
       <c r="B14" s="35">
         <v>5815118</v>
       </c>
@@ -1838,18 +1979,21 @@
       <c r="G14" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="H14" s="39">
+      <c r="H14" s="42">
+        <v>1</v>
+      </c>
+      <c r="I14" s="39">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="I14" s="40">
+      <c r="J14" s="40">
         <v>74</v>
       </c>
-      <c r="J14" s="41">
+      <c r="K14" s="41">
         <v>74</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="15.75">
+    <row r="15" spans="1:11" ht="15.6">
       <c r="B15" s="35">
         <v>10963297</v>
       </c>
@@ -1868,18 +2012,21 @@
       <c r="G15" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="H15" s="39">
+      <c r="H15" s="42">
+        <v>1</v>
+      </c>
+      <c r="I15" s="39">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="I15" s="40">
+      <c r="J15" s="40">
         <v>60</v>
       </c>
-      <c r="J15" s="41">
+      <c r="K15" s="41">
         <v>720</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="15.75">
+    <row r="16" spans="1:11" ht="15.6">
       <c r="B16" s="35">
         <v>10939665</v>
       </c>
@@ -1898,18 +2045,21 @@
       <c r="G16" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="H16" s="39">
+      <c r="H16" s="42">
+        <v>1</v>
+      </c>
+      <c r="I16" s="39">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="I16" s="40" t="s">
+      <c r="J16" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="J16" s="41">
+      <c r="K16" s="41">
         <v>392</v>
       </c>
     </row>
-    <row r="17" spans="2:10" ht="15.75">
+    <row r="17" spans="2:11" ht="15.6">
       <c r="B17" s="35">
         <v>10966256</v>
       </c>
@@ -1928,18 +2078,21 @@
       <c r="G17" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="H17" s="39">
+      <c r="H17" s="42">
+        <v>1</v>
+      </c>
+      <c r="I17" s="39">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="I17" s="40" t="s">
+      <c r="J17" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="J17" s="41">
+      <c r="K17" s="41">
         <v>632</v>
       </c>
     </row>
-    <row r="18" spans="2:10" ht="15.75">
+    <row r="18" spans="2:11" ht="15.6">
       <c r="B18" s="35">
         <v>10950272</v>
       </c>
@@ -1958,22 +2111,27 @@
       <c r="G18" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="H18" s="39">
+      <c r="H18" s="42">
+        <v>1</v>
+      </c>
+      <c r="I18" s="39">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="I18" s="40" t="s">
+      <c r="J18" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="J18" s="41">
+      <c r="K18" s="41">
         <v>990</v>
       </c>
     </row>
-    <row r="19" spans="2:10" ht="15.75">
+    <row r="19" spans="2:11" ht="15.6">
       <c r="B19" s="35">
         <v>10945337</v>
       </c>
-      <c r="C19" s="36"/>
+      <c r="C19" s="36">
+        <v>13970</v>
+      </c>
       <c r="D19" s="37">
         <v>45619</v>
       </c>
@@ -1986,42 +2144,49 @@
       <c r="G19" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="H19" s="39">
+      <c r="H19" s="42">
+        <v>1</v>
+      </c>
+      <c r="I19" s="39">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="I19" s="40" t="s">
+      <c r="J19" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="J19" s="41">
+      <c r="K19" s="41">
         <v>712</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B1:J19">
-    <filterColumn colId="2"/>
-    <filterColumn colId="5"/>
-  </autoFilter>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G19">
-      <formula1>'[1]ROOM TYPE'!$A$1:$A$24</formula1>
-    </dataValidation>
-  </dataValidations>
+  <autoFilter ref="B1:K19" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000000000000}">
+          <x14:formula1>
+            <xm:f>'D:\Hotels\Siva Golden Bay\Invoices DEC 24\New Till 28.12\[Anex-DEC till 28.xlsx]ROOM TYPE'!#REF!</xm:f>
+          </x14:formula1>
+          <xm:sqref>G2:G19</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:J57"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultRowHeight="13.2"/>
   <cols>
-    <col min="1" max="8" width="15.7109375" customWidth="1"/>
+    <col min="1" max="8" width="15.6640625" customWidth="1"/>
     <col min="9" max="9" width="24" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="17.25" thickTop="1" thickBot="1">
+    <row r="1" spans="1:10" ht="16.8" thickTop="1" thickBot="1">
       <c r="A1" s="11" t="s">
         <v>5</v>
       </c>
@@ -2053,7 +2218,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="15" thickTop="1">
+    <row r="2" spans="1:10" ht="14.4" thickTop="1">
       <c r="A2" s="14">
         <v>45413</v>
       </c>
@@ -2087,7 +2252,7 @@
         <v>64.5</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="14.25">
+    <row r="3" spans="1:10" ht="13.8">
       <c r="A3" s="17">
         <v>45423</v>
       </c>
@@ -2121,7 +2286,7 @@
         <v>58.5</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="14.25">
+    <row r="4" spans="1:10" ht="13.8">
       <c r="A4" s="17">
         <v>45474</v>
       </c>
@@ -2155,7 +2320,7 @@
         <v>55.5</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="14.25">
+    <row r="5" spans="1:10" ht="13.8">
       <c r="A5" s="17">
         <v>45505</v>
       </c>
@@ -2189,7 +2354,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="14.25">
+    <row r="6" spans="1:10" ht="13.8">
       <c r="A6" s="17">
         <v>45536</v>
       </c>
@@ -2223,7 +2388,7 @@
         <v>55.5</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="15" thickBot="1">
+    <row r="7" spans="1:10" ht="14.4" thickBot="1">
       <c r="A7" s="17">
         <v>45566</v>
       </c>
@@ -2257,7 +2422,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="15" thickTop="1">
+    <row r="8" spans="1:10" ht="14.4" thickTop="1">
       <c r="A8" s="14">
         <v>45597</v>
       </c>
@@ -2296,7 +2461,7 @@
         <v>73.5</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="14.25">
+    <row r="9" spans="1:10" ht="13.8">
       <c r="A9" s="17">
         <v>45612</v>
       </c>
@@ -2335,7 +2500,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="14.25">
+    <row r="10" spans="1:10" ht="13.8">
       <c r="A10" s="17">
         <v>45650</v>
       </c>
@@ -2374,7 +2539,7 @@
         <v>76.5</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="14.25">
+    <row r="11" spans="1:10" ht="13.8">
       <c r="A11" s="17">
         <v>45668</v>
       </c>
@@ -2413,7 +2578,7 @@
         <v>46.5</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="14.25">
+    <row r="12" spans="1:10" ht="13.8">
       <c r="A12" s="17">
         <v>45717</v>
       </c>
@@ -2451,7 +2616,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="14.25">
+    <row r="13" spans="1:10" ht="13.8">
       <c r="A13" s="17">
         <v>45740</v>
       </c>
@@ -2490,7 +2655,7 @@
         <v>58.5</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="14.25">
+    <row r="14" spans="1:10" ht="13.8">
       <c r="A14" s="17">
         <v>45756</v>
       </c>
@@ -2541,35 +2706,48 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I1">
-      <formula1>'[2]rate code'!$A$1:$A$15</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1:E1">
-      <formula1>'[3]ROOM TYPE'!$A$1:$A$24</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G1:H1">
-      <formula1>'[4]ROOM TYPE'!$A$1:$A$24</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0100-000000000000}">
+          <x14:formula1>
+            <xm:f>'C:\Users\Area-Credit2\AppData\Local\Microsoft\Windows\INetCache\Content.Outlook\R4F19B9Y\[biblio Globus.xls]rate code'!#REF!</xm:f>
+          </x14:formula1>
+          <xm:sqref>I1</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0100-000001000000}">
+          <x14:formula1>
+            <xm:f>'C:\Users\Area-Credit2\AppData\Local\Microsoft\Windows\INetCache\Content.Outlook\R4F19B9Y\[biblio -DEC.xlsx]ROOM TYPE'!#REF!</xm:f>
+          </x14:formula1>
+          <xm:sqref>C1:E1</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0100-000002000000}">
+          <x14:formula1>
+            <xm:f>'D:\Hotels\Siva Golden Bay\Invoices DEC 24\Biblio -Dec\[Copy of biblio -DEC (2).xlsx]ROOM TYPE'!#REF!</xm:f>
+          </x14:formula1>
+          <xm:sqref>G1:H1</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:J15"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultRowHeight="13.2"/>
   <cols>
-    <col min="1" max="1" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="8" width="15.7109375" customWidth="1"/>
+    <col min="1" max="1" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="8" width="15.6640625" customWidth="1"/>
     <col min="9" max="9" width="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="16.5" thickTop="1">
+    <row r="1" spans="1:10" ht="16.2" thickTop="1">
       <c r="A1" s="9" t="s">
         <v>5</v>
       </c>
@@ -2601,7 +2779,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="14.25">
+    <row r="2" spans="1:10" ht="13.8">
       <c r="A2" s="7">
         <v>45487</v>
       </c>
@@ -2636,7 +2814,7 @@
         <v>55.5</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="14.25">
+    <row r="3" spans="1:10" ht="13.8">
       <c r="A3" s="7">
         <v>45505</v>
       </c>
@@ -2672,7 +2850,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="14.25">
+    <row r="4" spans="1:10" ht="13.8">
       <c r="A4" s="7">
         <v>45536</v>
       </c>
@@ -2708,7 +2886,7 @@
         <v>49.5</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="15" thickBot="1">
+    <row r="5" spans="1:10" ht="14.4" thickBot="1">
       <c r="A5" s="7">
         <v>45566</v>
       </c>
@@ -2744,7 +2922,7 @@
         <v>55.5</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="15" thickTop="1">
+    <row r="6" spans="1:10" ht="14.4" thickTop="1">
       <c r="A6" s="14">
         <v>45597</v>
       </c>
@@ -2783,7 +2961,7 @@
         <v>73.5</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="14.25">
+    <row r="7" spans="1:10" ht="13.8">
       <c r="A7" s="17">
         <v>45612</v>
       </c>
@@ -2822,7 +3000,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="14.25">
+    <row r="8" spans="1:10" ht="13.8">
       <c r="A8" s="17">
         <v>45650</v>
       </c>
@@ -2861,7 +3039,7 @@
         <v>76.5</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="14.25">
+    <row r="9" spans="1:10" ht="13.8">
       <c r="A9" s="17">
         <v>45668</v>
       </c>
@@ -2900,7 +3078,7 @@
         <v>46.5</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="14.25">
+    <row r="10" spans="1:10" ht="13.8">
       <c r="A10" s="17">
         <v>45717</v>
       </c>
@@ -2938,7 +3116,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="14.25">
+    <row r="11" spans="1:10" ht="13.8">
       <c r="A11" s="17">
         <v>45740</v>
       </c>
@@ -2977,7 +3155,7 @@
         <v>58.5</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="14.25">
+    <row r="12" spans="1:10" ht="13.8">
       <c r="A12" s="17">
         <v>45756</v>
       </c>
@@ -3020,35 +3198,48 @@
       <c r="J15" s="23"/>
     </row>
   </sheetData>
-  <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I1">
-      <formula1>'[2]rate code'!$A$1:$A$15</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H1 C1:E1">
-      <formula1>'[3]ROOM TYPE'!$A$1:$A$24</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G1">
-      <formula1>'[4]ROOM TYPE'!$A$1:$A$24</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0200-000000000000}">
+          <x14:formula1>
+            <xm:f>'C:\Users\Area-Credit2\AppData\Local\Microsoft\Windows\INetCache\Content.Outlook\R4F19B9Y\[biblio Globus.xls]rate code'!#REF!</xm:f>
+          </x14:formula1>
+          <xm:sqref>I1</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0200-000001000000}">
+          <x14:formula1>
+            <xm:f>'C:\Users\Area-Credit2\AppData\Local\Microsoft\Windows\INetCache\Content.Outlook\R4F19B9Y\[biblio -DEC.xlsx]ROOM TYPE'!#REF!</xm:f>
+          </x14:formula1>
+          <xm:sqref>H1 C1:E1</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0200-000002000000}">
+          <x14:formula1>
+            <xm:f>'D:\Hotels\Siva Golden Bay\Invoices DEC 24\Biblio -Dec\[Copy of biblio -DEC (2).xlsx]ROOM TYPE'!#REF!</xm:f>
+          </x14:formula1>
+          <xm:sqref>G1</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:J8"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultRowHeight="13.2"/>
   <cols>
-    <col min="1" max="1" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="8" width="15.7109375" customWidth="1"/>
+    <col min="1" max="1" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="8" width="15.6640625" customWidth="1"/>
     <col min="9" max="9" width="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="16.5" thickTop="1">
+    <row r="1" spans="1:10" ht="16.2" thickTop="1">
       <c r="A1" s="9" t="s">
         <v>5</v>
       </c>
@@ -3080,7 +3271,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="14.25">
+    <row r="2" spans="1:10" ht="13.8">
       <c r="A2" s="7">
         <v>45577</v>
       </c>
@@ -3116,7 +3307,7 @@
         <v>55.5</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="14.25">
+    <row r="3" spans="1:10" ht="13.8">
       <c r="A3" s="7">
         <v>45597</v>
       </c>
@@ -3153,7 +3344,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="14.25">
+    <row r="4" spans="1:10" ht="13.8">
       <c r="A4" s="7">
         <v>45612</v>
       </c>
@@ -3192,7 +3383,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="14.25">
+    <row r="5" spans="1:10" ht="13.8">
       <c r="A5" s="7">
         <v>45650</v>
       </c>
@@ -3233,35 +3424,48 @@
       <c r="J8" s="23"/>
     </row>
   </sheetData>
-  <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I1">
-      <formula1>'[2]rate code'!$A$1:$A$15</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H1 C1:E1">
-      <formula1>'[3]ROOM TYPE'!$A$1:$A$24</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G1">
-      <formula1>'[4]ROOM TYPE'!$A$1:$A$24</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0300-000000000000}">
+          <x14:formula1>
+            <xm:f>'C:\Users\Area-Credit2\AppData\Local\Microsoft\Windows\INetCache\Content.Outlook\R4F19B9Y\[biblio Globus.xls]rate code'!#REF!</xm:f>
+          </x14:formula1>
+          <xm:sqref>I1</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0300-000001000000}">
+          <x14:formula1>
+            <xm:f>'C:\Users\Area-Credit2\AppData\Local\Microsoft\Windows\INetCache\Content.Outlook\R4F19B9Y\[biblio -DEC.xlsx]ROOM TYPE'!#REF!</xm:f>
+          </x14:formula1>
+          <xm:sqref>H1 C1:E1</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0300-000002000000}">
+          <x14:formula1>
+            <xm:f>'D:\Hotels\Siva Golden Bay\Invoices DEC 24\Biblio -Dec\[Copy of biblio -DEC (2).xlsx]ROOM TYPE'!#REF!</xm:f>
+          </x14:formula1>
+          <xm:sqref>G1</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:J17"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultRowHeight="13.2"/>
   <cols>
-    <col min="1" max="1" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="8" width="15.7109375" customWidth="1"/>
+    <col min="1" max="1" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="8" width="15.6640625" customWidth="1"/>
     <col min="9" max="9" width="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="16.5" thickTop="1">
+    <row r="1" spans="1:10" ht="16.2" thickTop="1">
       <c r="A1" s="9" t="s">
         <v>5</v>
       </c>
@@ -3293,7 +3497,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="14.25">
+    <row r="2" spans="1:10" ht="13.8">
       <c r="A2" s="7">
         <v>45612</v>
       </c>
@@ -3332,7 +3536,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="14.25">
+    <row r="3" spans="1:10" ht="13.8">
       <c r="A3" s="7">
         <v>45623</v>
       </c>
@@ -3369,7 +3573,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="14.25">
+    <row r="4" spans="1:10" ht="13.8">
       <c r="A4" s="7">
         <v>45650</v>
       </c>
@@ -3406,7 +3610,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="14.25">
+    <row r="5" spans="1:10" ht="13.8">
       <c r="A5" s="7">
         <v>45657</v>
       </c>
@@ -3445,7 +3649,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="14.25">
+    <row r="6" spans="1:10" ht="13.8">
       <c r="A6" s="7">
         <v>45658</v>
       </c>
@@ -3482,7 +3686,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="14.25">
+    <row r="7" spans="1:10" ht="13.8">
       <c r="A7" s="7">
         <v>45668</v>
       </c>
@@ -3526,19 +3730,32 @@
       <c r="I17" s="27"/>
     </row>
   </sheetData>
-  <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I1">
-      <formula1>'[2]rate code'!$A$1:$A$15</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H1 C1:E1">
-      <formula1>'[3]ROOM TYPE'!$A$1:$A$24</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G1">
-      <formula1>'[4]ROOM TYPE'!$A$1:$A$24</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0400-000000000000}">
+          <x14:formula1>
+            <xm:f>'C:\Users\Area-Credit2\AppData\Local\Microsoft\Windows\INetCache\Content.Outlook\R4F19B9Y\[biblio Globus.xls]rate code'!#REF!</xm:f>
+          </x14:formula1>
+          <xm:sqref>I1</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0400-000001000000}">
+          <x14:formula1>
+            <xm:f>'C:\Users\Area-Credit2\AppData\Local\Microsoft\Windows\INetCache\Content.Outlook\R4F19B9Y\[biblio -DEC.xlsx]ROOM TYPE'!#REF!</xm:f>
+          </x14:formula1>
+          <xm:sqref>H1 C1:E1</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0400-000002000000}">
+          <x14:formula1>
+            <xm:f>'D:\Hotels\Siva Golden Bay\Invoices DEC 24\Biblio -Dec\[Copy of biblio -DEC (2).xlsx]ROOM TYPE'!#REF!</xm:f>
+          </x14:formula1>
+          <xm:sqref>G1</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
</xml_diff>